<commit_message>
docs: finalize API testing submission artifacts
</commit_message>
<xml_diff>
--- a/submit/test-cases/member-4.xlsx
+++ b/submit/test-cases/member-4.xlsx
@@ -228,12 +228,12 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-001 — auth</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -243,7 +243,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -325,12 +325,12 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-002 — auth</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -340,7 +340,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -422,12 +422,12 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-003 — auth</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -437,7 +437,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -519,12 +519,12 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-004 — schema</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -534,7 +534,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -616,12 +616,12 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-005 — identity</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -713,12 +713,12 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-006 — repeat</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -810,12 +810,12 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-007 — auth</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -825,7 +825,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -907,12 +907,12 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-008 — security</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -922,7 +922,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -1004,12 +1004,12 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-009 — privacy</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -1101,12 +1101,12 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-010 — idor</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -1198,12 +1198,12 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-011 — positive</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -1295,12 +1295,12 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-012 — positive</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1310,7 +1310,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -1392,12 +1392,12 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-013 — positive</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1407,7 +1407,7 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -1489,12 +1489,12 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-014 — positive</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -1586,12 +1586,12 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-015 — boundary</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -1601,7 +1601,7 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -1683,12 +1683,12 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-016 — boundary</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -1780,12 +1780,12 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-017 — boundary</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -1795,7 +1795,7 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -1877,12 +1877,12 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-018 — boundary</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -1892,7 +1892,7 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -1974,12 +1974,12 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-019 — boundary</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -1989,7 +1989,7 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -2071,12 +2071,12 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-020 — boundary</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -2086,7 +2086,7 @@
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -2168,12 +2168,12 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-021 — boundary</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -2265,12 +2265,12 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-022 — boundary</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -2280,7 +2280,7 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -2362,12 +2362,12 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-023 — boundary</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -2459,12 +2459,12 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-024 — type</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -2556,12 +2556,12 @@
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-025 — boundary</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -2571,7 +2571,7 @@
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -2653,12 +2653,12 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-026 — boundary</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -2668,7 +2668,7 @@
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -2750,12 +2750,12 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-027 — boundary</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -2765,7 +2765,7 @@
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -2847,12 +2847,12 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-028 — boundary</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -2862,7 +2862,7 @@
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -2944,12 +2944,12 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-029 — security</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -2959,7 +2959,7 @@
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -3041,12 +3041,12 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-030 — boundary</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -3138,12 +3138,12 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-031 — type</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -3153,7 +3153,7 @@
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -3235,12 +3235,12 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-032 — type</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -3250,7 +3250,7 @@
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -3332,12 +3332,12 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-033 — auth</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -3429,12 +3429,12 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-034 — auth</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -3444,7 +3444,7 @@
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -3526,22 +3526,22 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-035 — security</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">BUG-04-001</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../evidence/BUG-04-001.png</t>
         </is>
       </c>
     </row>
@@ -3623,12 +3623,12 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-036 — security</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -3638,7 +3638,7 @@
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -3720,12 +3720,12 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-037 — security</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -3735,7 +3735,7 @@
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -3817,12 +3817,12 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-038 — security</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -3832,7 +3832,7 @@
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -3914,12 +3914,12 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-039 — security</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -3929,7 +3929,7 @@
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -4011,12 +4011,12 @@
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-040 — schema</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -4026,7 +4026,7 @@
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -4108,12 +4108,12 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-041 — human-security</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
@@ -4123,7 +4123,7 @@
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -4205,12 +4205,12 @@
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-042 — human-security</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -4220,7 +4220,7 @@
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -4302,12 +4302,12 @@
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-043 — human-security</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
@@ -4317,7 +4317,7 @@
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -4399,12 +4399,12 @@
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-044 — human-security</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -4496,12 +4496,12 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR04-045 — human-security</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
@@ -4511,7 +4511,7 @@
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -4593,12 +4593,12 @@
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-001 — state-matrix</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
@@ -4608,7 +4608,7 @@
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -4690,12 +4690,12 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-002 — state-matrix</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; FAIL</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
@@ -4705,7 +4705,7 @@
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -4787,12 +4787,12 @@
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-003 — state-matrix</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
@@ -4802,7 +4802,7 @@
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -4884,12 +4884,12 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-004 — state-matrix</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
@@ -4899,7 +4899,7 @@
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -4981,12 +4981,12 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-005 — state-matrix</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; FAIL</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
@@ -4996,7 +4996,7 @@
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -5078,12 +5078,12 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-006 — state-matrix</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
@@ -5093,7 +5093,7 @@
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -5175,12 +5175,12 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-007 — state-matrix</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -5272,12 +5272,12 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-008 — state-matrix</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; FAIL</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
@@ -5287,7 +5287,7 @@
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -5369,12 +5369,12 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-009 — state-matrix</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -5384,7 +5384,7 @@
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -5466,12 +5466,12 @@
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-010 — state-matrix</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; FAIL</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
@@ -5481,7 +5481,7 @@
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -5563,12 +5563,12 @@
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-011 — state-matrix</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -5578,7 +5578,7 @@
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -5660,12 +5660,12 @@
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-012 — state-matrix</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -5675,7 +5675,7 @@
       </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -5757,12 +5757,12 @@
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-013 — state-matrix</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
@@ -5772,7 +5772,7 @@
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -5854,12 +5854,12 @@
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-014 — state-matrix</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; FAIL</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
@@ -5869,7 +5869,7 @@
       </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -5951,12 +5951,12 @@
       </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-015 — state-matrix</t>
         </is>
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
@@ -5966,7 +5966,7 @@
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -6048,12 +6048,12 @@
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-016 — state-matrix</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
@@ -6063,7 +6063,7 @@
       </c>
       <c r="S62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -6145,12 +6145,12 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-017 — state-matrix</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="S63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -6242,12 +6242,12 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-018 — state-matrix</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
@@ -6257,7 +6257,7 @@
       </c>
       <c r="S64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -6339,12 +6339,12 @@
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-019 — state-matrix</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
@@ -6354,7 +6354,7 @@
       </c>
       <c r="S65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -6436,12 +6436,12 @@
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-020 — state-matrix</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
@@ -6451,7 +6451,7 @@
       </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -6533,12 +6533,12 @@
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-021 — state-matrix</t>
         </is>
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
@@ -6548,7 +6548,7 @@
       </c>
       <c r="S67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -6630,12 +6630,12 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-022 — state-matrix</t>
         </is>
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
@@ -6645,7 +6645,7 @@
       </c>
       <c r="S68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -6727,12 +6727,12 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-023 — state-matrix</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
@@ -6742,7 +6742,7 @@
       </c>
       <c r="S69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -6824,12 +6824,12 @@
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-024 — state-matrix</t>
         </is>
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R70" t="inlineStr">
@@ -6839,7 +6839,7 @@
       </c>
       <c r="S70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -6921,12 +6921,12 @@
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-025 — state-matrix</t>
         </is>
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
@@ -6936,7 +6936,7 @@
       </c>
       <c r="S71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -7018,12 +7018,12 @@
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-026 — cancel/ownership</t>
         </is>
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
@@ -7033,7 +7033,7 @@
       </c>
       <c r="S72" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -7115,12 +7115,12 @@
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-027 — cancel/ownership</t>
         </is>
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; FAIL</t>
         </is>
       </c>
       <c r="R73" t="inlineStr">
@@ -7130,7 +7130,7 @@
       </c>
       <c r="S73" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -7212,12 +7212,12 @@
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-028 — cancel/ownership</t>
         </is>
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R74" t="inlineStr">
@@ -7227,7 +7227,7 @@
       </c>
       <c r="S74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -7309,12 +7309,12 @@
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-029 — cancel/ownership</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R75" t="inlineStr">
@@ -7324,7 +7324,7 @@
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -7406,12 +7406,12 @@
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-030 — cancel/ownership</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R76" t="inlineStr">
@@ -7421,7 +7421,7 @@
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -7503,12 +7503,12 @@
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-031 — cancel/ownership</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; FAIL</t>
         </is>
       </c>
       <c r="R77" t="inlineStr">
@@ -7518,7 +7518,7 @@
       </c>
       <c r="S77" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -7600,12 +7600,12 @@
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-032 — cancel/ownership</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; FAIL</t>
         </is>
       </c>
       <c r="R78" t="inlineStr">
@@ -7615,7 +7615,7 @@
       </c>
       <c r="S78" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -7697,12 +7697,12 @@
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-033 — auth-negative</t>
         </is>
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; FAIL</t>
         </is>
       </c>
       <c r="R79" t="inlineStr">
@@ -7712,7 +7712,7 @@
       </c>
       <c r="S79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -7794,12 +7794,12 @@
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-034 — auth-negative</t>
         </is>
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; FAIL</t>
         </is>
       </c>
       <c r="R80" t="inlineStr">
@@ -7809,7 +7809,7 @@
       </c>
       <c r="S80" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -7891,12 +7891,12 @@
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-035 — auth-negative</t>
         </is>
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; FAIL</t>
         </is>
       </c>
       <c r="R81" t="inlineStr">
@@ -7906,7 +7906,7 @@
       </c>
       <c r="S81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -7988,12 +7988,12 @@
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-036 — auth-negative</t>
         </is>
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; FAIL</t>
         </is>
       </c>
       <c r="R82" t="inlineStr">
@@ -8003,7 +8003,7 @@
       </c>
       <c r="S82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -8085,12 +8085,12 @@
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-037 — auth-negative</t>
         </is>
       </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; FAIL</t>
         </is>
       </c>
       <c r="R83" t="inlineStr">
@@ -8100,7 +8100,7 @@
       </c>
       <c r="S83" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -8182,12 +8182,12 @@
       </c>
       <c r="P84" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-038 — auth-negative</t>
         </is>
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; FAIL</t>
         </is>
       </c>
       <c r="R84" t="inlineStr">
@@ -8197,7 +8197,7 @@
       </c>
       <c r="S84" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -8279,12 +8279,12 @@
       </c>
       <c r="P85" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-039 — auth-negative</t>
         </is>
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; FAIL</t>
         </is>
       </c>
       <c r="R85" t="inlineStr">
@@ -8294,7 +8294,7 @@
       </c>
       <c r="S85" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -8376,12 +8376,12 @@
       </c>
       <c r="P86" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-040 — auth-negative</t>
         </is>
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R86" t="inlineStr">
@@ -8391,7 +8391,7 @@
       </c>
       <c r="S86" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -8473,12 +8473,12 @@
       </c>
       <c r="P87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-041 — auth-negative</t>
         </is>
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R87" t="inlineStr">
@@ -8488,7 +8488,7 @@
       </c>
       <c r="S87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -8570,12 +8570,12 @@
       </c>
       <c r="P88" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-042 — auth-negative</t>
         </is>
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R88" t="inlineStr">
@@ -8585,7 +8585,7 @@
       </c>
       <c r="S88" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -8667,12 +8667,12 @@
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-043 — auth-negative</t>
         </is>
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R89" t="inlineStr">
@@ -8682,7 +8682,7 @@
       </c>
       <c r="S89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -8764,12 +8764,12 @@
       </c>
       <c r="P90" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-044 — auth-negative</t>
         </is>
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R90" t="inlineStr">
@@ -8779,7 +8779,7 @@
       </c>
       <c r="S90" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -8861,12 +8861,12 @@
       </c>
       <c r="P91" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-045 — auth-negative</t>
         </is>
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R91" t="inlineStr">
@@ -8876,7 +8876,7 @@
       </c>
       <c r="S91" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -8958,12 +8958,12 @@
       </c>
       <c r="P92" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-046 — human-state-security</t>
         </is>
       </c>
       <c r="Q92" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R92" t="inlineStr">
@@ -8973,7 +8973,7 @@
       </c>
       <c r="S92" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -9055,12 +9055,12 @@
       </c>
       <c r="P93" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-047 — human-state-security</t>
         </is>
       </c>
       <c r="Q93" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R93" t="inlineStr">
@@ -9070,7 +9070,7 @@
       </c>
       <c r="S93" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -9152,12 +9152,12 @@
       </c>
       <c r="P94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-048 — human-state-security</t>
         </is>
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R94" t="inlineStr">
@@ -9167,7 +9167,7 @@
       </c>
       <c r="S94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -9249,12 +9249,12 @@
       </c>
       <c r="P95" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-049 — human-state-security</t>
         </is>
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R95" t="inlineStr">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="S95" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -9346,12 +9346,12 @@
       </c>
       <c r="P96" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR10-050 — human-state-security</t>
         </is>
       </c>
       <c r="Q96" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 400; PASS</t>
         </is>
       </c>
       <c r="R96" t="inlineStr">
@@ -9361,7 +9361,7 @@
       </c>
       <c r="S96" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -9443,12 +9443,12 @@
       </c>
       <c r="P97" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-001 — list</t>
         </is>
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R97" t="inlineStr">
@@ -9458,7 +9458,7 @@
       </c>
       <c r="S97" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -9540,12 +9540,12 @@
       </c>
       <c r="P98" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-002 — auth</t>
         </is>
       </c>
       <c r="Q98" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R98" t="inlineStr">
@@ -9555,7 +9555,7 @@
       </c>
       <c r="S98" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -9637,12 +9637,12 @@
       </c>
       <c r="P99" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-003 — auth</t>
         </is>
       </c>
       <c r="Q99" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R99" t="inlineStr">
@@ -9652,7 +9652,7 @@
       </c>
       <c r="S99" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -9734,22 +9734,22 @@
       </c>
       <c r="P100" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-004 — auth</t>
         </is>
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R100" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">BUG-04-005</t>
         </is>
       </c>
       <c r="S100" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../evidence/BUG-04-005.png</t>
         </is>
       </c>
     </row>
@@ -9831,12 +9831,12 @@
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-005 — auth</t>
         </is>
       </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R101" t="inlineStr">
@@ -9846,7 +9846,7 @@
       </c>
       <c r="S101" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -9928,12 +9928,12 @@
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-006 — schema</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R102" t="inlineStr">
@@ -9943,7 +9943,7 @@
       </c>
       <c r="S102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -10025,12 +10025,12 @@
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-007 — privacy</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R103" t="inlineStr">
@@ -10040,7 +10040,7 @@
       </c>
       <c r="S103" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -10122,12 +10122,12 @@
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-008 — privacy</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R104" t="inlineStr">
@@ -10137,7 +10137,7 @@
       </c>
       <c r="S104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -10219,12 +10219,12 @@
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-009 — schema</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R105" t="inlineStr">
@@ -10234,7 +10234,7 @@
       </c>
       <c r="S105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -10316,12 +10316,12 @@
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-010 — schema</t>
         </is>
       </c>
       <c r="Q106" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R106" t="inlineStr">
@@ -10331,7 +10331,7 @@
       </c>
       <c r="S106" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -10413,12 +10413,12 @@
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-011 — idor</t>
         </is>
       </c>
       <c r="Q107" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R107" t="inlineStr">
@@ -10428,7 +10428,7 @@
       </c>
       <c r="S107" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -10510,12 +10510,12 @@
       </c>
       <c r="P108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-012 — repeat</t>
         </is>
       </c>
       <c r="Q108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R108" t="inlineStr">
@@ -10525,7 +10525,7 @@
       </c>
       <c r="S108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -10607,12 +10607,12 @@
       </c>
       <c r="P109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-013 — positive</t>
         </is>
       </c>
       <c r="Q109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R109" t="inlineStr">
@@ -10622,7 +10622,7 @@
       </c>
       <c r="S109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -10704,12 +10704,12 @@
       </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-014 — positive</t>
         </is>
       </c>
       <c r="Q110" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R110" t="inlineStr">
@@ -10719,7 +10719,7 @@
       </c>
       <c r="S110" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -10801,12 +10801,12 @@
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-015 — negative</t>
         </is>
       </c>
       <c r="Q111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R111" t="inlineStr">
@@ -10816,7 +10816,7 @@
       </c>
       <c r="S111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -10898,12 +10898,12 @@
       </c>
       <c r="P112" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-016 — negative</t>
         </is>
       </c>
       <c r="Q112" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R112" t="inlineStr">
@@ -10913,7 +10913,7 @@
       </c>
       <c r="S112" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -10995,12 +10995,12 @@
       </c>
       <c r="P113" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-017 — negative</t>
         </is>
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R113" t="inlineStr">
@@ -11010,7 +11010,7 @@
       </c>
       <c r="S113" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -11092,12 +11092,12 @@
       </c>
       <c r="P114" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-018 — negative</t>
         </is>
       </c>
       <c r="Q114" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R114" t="inlineStr">
@@ -11107,7 +11107,7 @@
       </c>
       <c r="S114" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -11189,12 +11189,12 @@
       </c>
       <c r="P115" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-019 — negative</t>
         </is>
       </c>
       <c r="Q115" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R115" t="inlineStr">
@@ -11204,7 +11204,7 @@
       </c>
       <c r="S115" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -11286,12 +11286,12 @@
       </c>
       <c r="P116" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-020 — negative</t>
         </is>
       </c>
       <c r="Q116" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R116" t="inlineStr">
@@ -11301,7 +11301,7 @@
       </c>
       <c r="S116" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -11383,12 +11383,12 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-021 — repeat</t>
         </is>
       </c>
       <c r="Q117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R117" t="inlineStr">
@@ -11398,7 +11398,7 @@
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -11480,12 +11480,12 @@
       </c>
       <c r="P118" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-022 — auth</t>
         </is>
       </c>
       <c r="Q118" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R118" t="inlineStr">
@@ -11495,7 +11495,7 @@
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -11577,12 +11577,12 @@
       </c>
       <c r="P119" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-023 — auth</t>
         </is>
       </c>
       <c r="Q119" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R119" t="inlineStr">
@@ -11592,7 +11592,7 @@
       </c>
       <c r="S119" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -11674,12 +11674,12 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-024 — auth</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R120" t="inlineStr">
@@ -11689,7 +11689,7 @@
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -11771,12 +11771,12 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-025 — auth</t>
         </is>
       </c>
       <c r="Q121" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R121" t="inlineStr">
@@ -11786,7 +11786,7 @@
       </c>
       <c r="S121" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -11868,12 +11868,12 @@
       </c>
       <c r="P122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-026 — idor</t>
         </is>
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R122" t="inlineStr">
@@ -11883,7 +11883,7 @@
       </c>
       <c r="S122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -11965,22 +11965,22 @@
       </c>
       <c r="P123" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-027 — self-delete</t>
         </is>
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R123" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">BUG-04-006</t>
         </is>
       </c>
       <c r="S123" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../evidence/BUG-04-006.png</t>
         </is>
       </c>
     </row>
@@ -12062,12 +12062,12 @@
       </c>
       <c r="P124" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-028 — schema</t>
         </is>
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R124" t="inlineStr">
@@ -12077,7 +12077,7 @@
       </c>
       <c r="S124" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -12159,12 +12159,12 @@
       </c>
       <c r="P125" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-029 — schema</t>
         </is>
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R125" t="inlineStr">
@@ -12174,7 +12174,7 @@
       </c>
       <c r="S125" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -12256,12 +12256,12 @@
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-030 — privacy</t>
         </is>
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R126" t="inlineStr">
@@ -12271,7 +12271,7 @@
       </c>
       <c r="S126" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -12353,12 +12353,12 @@
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-031 — integrity</t>
         </is>
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R127" t="inlineStr">
@@ -12368,7 +12368,7 @@
       </c>
       <c r="S127" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -12450,12 +12450,12 @@
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-032 — type</t>
         </is>
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R128" t="inlineStr">
@@ -12465,7 +12465,7 @@
       </c>
       <c r="S128" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -12547,12 +12547,12 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-033 — security</t>
         </is>
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R129" t="inlineStr">
@@ -12562,7 +12562,7 @@
       </c>
       <c r="S129" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -12644,12 +12644,12 @@
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-034 — security</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
@@ -12659,7 +12659,7 @@
       </c>
       <c r="S130" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -12741,12 +12741,12 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-035 — privacy</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
@@ -12756,7 +12756,7 @@
       </c>
       <c r="S131" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -12838,12 +12838,12 @@
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-036 — authorization</t>
         </is>
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
@@ -12853,7 +12853,7 @@
       </c>
       <c r="S132" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -12935,12 +12935,12 @@
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-037 — authorization</t>
         </is>
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R133" t="inlineStr">
@@ -12950,7 +12950,7 @@
       </c>
       <c r="S133" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -13032,12 +13032,12 @@
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-038 — concurrency</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R134" t="inlineStr">
@@ -13047,7 +13047,7 @@
       </c>
       <c r="S134" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -13129,12 +13129,12 @@
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-039 — schema</t>
         </is>
       </c>
       <c r="Q135" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; PASS</t>
         </is>
       </c>
       <c r="R135" t="inlineStr">
@@ -13144,7 +13144,7 @@
       </c>
       <c r="S135" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -13226,12 +13226,12 @@
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-040 — negative</t>
         </is>
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R136" t="inlineStr">
@@ -13241,7 +13241,7 @@
       </c>
       <c r="S136" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -13323,12 +13323,12 @@
       </c>
       <c r="P137" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-041 — human-security</t>
         </is>
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R137" t="inlineStr">
@@ -13338,7 +13338,7 @@
       </c>
       <c r="S137" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -13420,12 +13420,12 @@
       </c>
       <c r="P138" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-042 — human-security</t>
         </is>
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R138" t="inlineStr">
@@ -13435,7 +13435,7 @@
       </c>
       <c r="S138" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -13517,12 +13517,12 @@
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-043 — human-security</t>
         </is>
       </c>
       <c r="Q139" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R139" t="inlineStr">
@@ -13532,7 +13532,7 @@
       </c>
       <c r="S139" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -13614,12 +13614,12 @@
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-044 — human-security</t>
         </is>
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R140" t="inlineStr">
@@ -13629,7 +13629,7 @@
       </c>
       <c r="S140" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>
@@ -13711,12 +13711,12 @@
       </c>
       <c r="P141" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending Newman mapping</t>
+          <t xml:space="preserve">FR19-045 — human-security</t>
         </is>
       </c>
       <c r="Q141" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed</t>
+          <t xml:space="preserve">HTTP 200; FAIL</t>
         </is>
       </c>
       <c r="R141" t="inlineStr">
@@ -13726,7 +13726,7 @@
       </c>
       <c r="S141" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending authentic evidence</t>
+          <t xml:space="preserve">../newman/member-4/newman-full-report.html</t>
         </is>
       </c>
     </row>

</xml_diff>